<commit_message>
update registrasi dan integrasi rfid
</commit_message>
<xml_diff>
--- a/template excel data siman.xlsx
+++ b/template excel data siman.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\xampp_74\htdocs\ugtapetracking\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2421A3C-872F-406D-894A-79B35F295214}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33B99B97-63FF-4642-83BC-879D8F9CB383}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BEDAB03C-CF3C-604A-97F9-819FE9571DA0}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="117">
   <si>
     <t>No</t>
   </si>
@@ -379,6 +379,9 @@
   </si>
   <si>
     <t>Tape 20</t>
+  </si>
+  <si>
+    <t>dob</t>
   </si>
 </sst>
 </file>
@@ -788,7 +791,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6774A036-93D0-9A46-814F-52ECCE9530C0}">
-  <dimension ref="A1:BX21"/>
+  <dimension ref="A1:BY21"/>
   <sheetFormatPr defaultColWidth="10.81640625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7.36328125" style="1" bestFit="1" customWidth="1"/>
@@ -866,10 +869,11 @@
     <col min="74" max="74" width="15.453125" style="1" bestFit="1" customWidth="1"/>
     <col min="75" max="75" width="18" style="1" bestFit="1" customWidth="1"/>
     <col min="76" max="76" width="16.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="77" max="16384" width="10.81640625" style="1"/>
+    <col min="77" max="77" width="14.453125" style="4" customWidth="1"/>
+    <col min="78" max="16384" width="10.81640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:76">
+    <row r="1" spans="1:77">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1098,8 +1102,11 @@
       <c r="BX1" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="2" spans="1:76">
+      <c r="BY1" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2" spans="1:77">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1138,8 +1145,11 @@
       </c>
       <c r="BW2" s="2"/>
       <c r="BX2" s="2"/>
-    </row>
-    <row r="3" spans="1:76">
+      <c r="BY2" s="4">
+        <v>33527</v>
+      </c>
+    </row>
+    <row r="3" spans="1:77">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1173,8 +1183,11 @@
       <c r="BN3" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:76">
+      <c r="BY3" s="4">
+        <v>33528</v>
+      </c>
+    </row>
+    <row r="4" spans="1:77">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1208,8 +1221,11 @@
       <c r="BN4" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:76">
+      <c r="BY4" s="4">
+        <v>33529</v>
+      </c>
+    </row>
+    <row r="5" spans="1:77">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1243,8 +1259,11 @@
       <c r="BN5" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:76">
+      <c r="BY5" s="4">
+        <v>33530</v>
+      </c>
+    </row>
+    <row r="6" spans="1:77">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1278,8 +1297,11 @@
       <c r="BN6" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="7" spans="1:76">
+      <c r="BY6" s="4">
+        <v>33531</v>
+      </c>
+    </row>
+    <row r="7" spans="1:77">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1313,8 +1335,11 @@
       <c r="BN7" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="8" spans="1:76">
+      <c r="BY7" s="4">
+        <v>33532</v>
+      </c>
+    </row>
+    <row r="8" spans="1:77">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1348,8 +1373,11 @@
       <c r="BN8" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:76">
+      <c r="BY8" s="4">
+        <v>33533</v>
+      </c>
+    </row>
+    <row r="9" spans="1:77">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1383,8 +1411,11 @@
       <c r="BN9" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:76">
+      <c r="BY9" s="4">
+        <v>33534</v>
+      </c>
+    </row>
+    <row r="10" spans="1:77">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1418,8 +1449,11 @@
       <c r="BN10" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:76">
+      <c r="BY10" s="4">
+        <v>33535</v>
+      </c>
+    </row>
+    <row r="11" spans="1:77">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1453,8 +1487,11 @@
       <c r="BN11" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:76">
+      <c r="BY11" s="4">
+        <v>33536</v>
+      </c>
+    </row>
+    <row r="12" spans="1:77">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1488,8 +1525,11 @@
       <c r="BN12" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:76">
+      <c r="BY12" s="4">
+        <v>33537</v>
+      </c>
+    </row>
+    <row r="13" spans="1:77">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1523,8 +1563,11 @@
       <c r="BN13" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:76">
+      <c r="BY13" s="4">
+        <v>33538</v>
+      </c>
+    </row>
+    <row r="14" spans="1:77">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1558,8 +1601,11 @@
       <c r="BN14" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:76">
+      <c r="BY14" s="4">
+        <v>33539</v>
+      </c>
+    </row>
+    <row r="15" spans="1:77">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1593,8 +1639,11 @@
       <c r="BN15" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:76">
+      <c r="BY15" s="4">
+        <v>33540</v>
+      </c>
+    </row>
+    <row r="16" spans="1:77">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -1628,8 +1677,11 @@
       <c r="BN16" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:66">
+      <c r="BY16" s="4">
+        <v>33541</v>
+      </c>
+    </row>
+    <row r="17" spans="1:77">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -1663,8 +1715,11 @@
       <c r="BN17" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:66">
+      <c r="BY17" s="4">
+        <v>33542</v>
+      </c>
+    </row>
+    <row r="18" spans="1:77">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -1698,8 +1753,11 @@
       <c r="BN18" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:66">
+      <c r="BY18" s="4">
+        <v>33543</v>
+      </c>
+    </row>
+    <row r="19" spans="1:77">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -1733,8 +1791,11 @@
       <c r="BN19" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:66">
+      <c r="BY19" s="4">
+        <v>33544</v>
+      </c>
+    </row>
+    <row r="20" spans="1:77">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -1768,8 +1829,11 @@
       <c r="BN20" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:66">
+      <c r="BY20" s="4">
+        <v>33545</v>
+      </c>
+    </row>
+    <row r="21" spans="1:77">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -1802,6 +1866,9 @@
       </c>
       <c r="BN21" s="2">
         <v>1</v>
+      </c>
+      <c r="BY21" s="4">
+        <v>33546</v>
       </c>
     </row>
   </sheetData>

</xml_diff>